<commit_message>
feat: add new fields to migration template and include extra inspection and order data in database import
</commit_message>
<xml_diff>
--- a/Plantilla_Migracion_Azkell.xlsx
+++ b/Plantilla_Migracion_Azkell.xlsx
@@ -447,7 +447,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:K1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -474,10 +474,19 @@
       <c r="H1" t="str">
         <v>Supervisor</v>
       </c>
+      <c r="I1" t="str">
+        <v>Motivo</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Situacion Inicial</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Comentario Cierre</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -546,7 +555,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:I1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -567,10 +576,19 @@
       <c r="F1" t="str">
         <v>Observaciones Generales</v>
       </c>
+      <c r="G1" t="str">
+        <v>Estado Llantas</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Estado Frenos</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Estado Luces</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>